<commit_message>
refactor: add method to filter and exclude DSR cluster dataframe based on act_price_da minor fix on raiso error message for filter on dsr_type
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/dsr/dsr_cluster_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/dsr/dsr_cluster_2030.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ITca</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2170,19 +2170,19 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>36.745</v>
+        <v>40</v>
       </c>
       <c r="F40" t="n">
         <v>24</v>
       </c>
       <c r="G40" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H40" t="n">
-        <v>-1</v>
+        <v>500</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ITcn</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>188.976</v>
+        <v>10</v>
       </c>
       <c r="F41" t="n">
         <v>24</v>
@@ -2223,7 +2223,7 @@
         <v>24</v>
       </c>
       <c r="H41" t="n">
-        <v>-1</v>
+        <v>150</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
@@ -2244,12 +2244,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ITcs</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>191.601</v>
+        <v>20</v>
       </c>
       <c r="F42" t="n">
         <v>24</v>
@@ -2267,7 +2267,7 @@
         <v>24</v>
       </c>
       <c r="H42" t="n">
-        <v>-1</v>
+        <v>200</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
@@ -2288,12 +2288,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ITn</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR3</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1428.696</v>
+        <v>40</v>
       </c>
       <c r="F43" t="n">
         <v>24</v>
@@ -2311,7 +2311,7 @@
         <v>24</v>
       </c>
       <c r="H43" t="n">
-        <v>-1</v>
+        <v>300</v>
       </c>
       <c r="I43" t="n">
         <v>1</v>
@@ -2332,12 +2332,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ITs</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR4</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2346,7 +2346,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>99.738</v>
+        <v>80</v>
       </c>
       <c r="F44" t="n">
         <v>24</v>
@@ -2355,7 +2355,7 @@
         <v>24</v>
       </c>
       <c r="H44" t="n">
-        <v>-1</v>
+        <v>500</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ITsar</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2390,19 +2390,19 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>10.499</v>
+        <v>328</v>
       </c>
       <c r="F45" t="n">
         <v>24</v>
       </c>
       <c r="G45" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H45" t="n">
-        <v>-1</v>
+        <v>300</v>
       </c>
       <c r="I45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2411,7 +2411,7 @@
         <v>1</v>
       </c>
       <c r="L45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2420,12 +2420,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ITsic</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2434,19 +2434,19 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>43.745</v>
+        <v>184</v>
       </c>
       <c r="F46" t="n">
         <v>24</v>
       </c>
       <c r="G46" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H46" t="n">
-        <v>-1</v>
+        <v>500</v>
       </c>
       <c r="I46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2455,7 +2455,7 @@
         <v>1</v>
       </c>
       <c r="L46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR3</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2478,20 +2478,20 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>40</v>
+        <v>593</v>
       </c>
       <c r="F47" t="n">
         <v>24</v>
       </c>
       <c r="G47" t="n">
+        <v>6</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I47" t="n">
         <v>4</v>
       </c>
-      <c r="H47" t="n">
-        <v>500</v>
-      </c>
-      <c r="I47" t="n">
-        <v>7</v>
-      </c>
       <c r="J47" t="n">
         <v>0</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>1</v>
       </c>
       <c r="L47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>10</v>
+        <v>64.70699999999999</v>
       </c>
       <c r="F48" t="n">
         <v>24</v>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>20</v>
+        <v>64.70699999999999</v>
       </c>
       <c r="F49" t="n">
         <v>24</v>
@@ -2575,7 +2575,7 @@
         <v>24</v>
       </c>
       <c r="H49" t="n">
-        <v>200</v>
+        <v>244</v>
       </c>
       <c r="I49" t="n">
         <v>1</v>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>SE1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>40</v>
+        <v>64.70699999999999</v>
       </c>
       <c r="F50" t="n">
         <v>24</v>
@@ -2619,7 +2619,7 @@
         <v>24</v>
       </c>
       <c r="H50" t="n">
-        <v>300</v>
+        <v>376</v>
       </c>
       <c r="I50" t="n">
         <v>1</v>
@@ -2640,12 +2640,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>SE2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DSR4</t>
+          <t>DSR1</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2654,7 +2654,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>80</v>
+        <v>91.36199999999999</v>
       </c>
       <c r="F51" t="n">
         <v>24</v>
@@ -2663,7 +2663,7 @@
         <v>24</v>
       </c>
       <c r="H51" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="I51" t="n">
         <v>1</v>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>SE2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2698,19 +2698,19 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>328</v>
+        <v>91.36199999999999</v>
       </c>
       <c r="F52" t="n">
         <v>24</v>
       </c>
       <c r="G52" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="H52" t="n">
-        <v>300</v>
+        <v>244</v>
       </c>
       <c r="I52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
         <v>1</v>
       </c>
       <c r="L52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2728,12 +2728,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>SE2</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DSR2</t>
+          <t>DSR3</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2742,19 +2742,19 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>184</v>
+        <v>91.36199999999999</v>
       </c>
       <c r="F53" t="n">
         <v>24</v>
       </c>
       <c r="G53" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="H53" t="n">
-        <v>500</v>
+        <v>376</v>
       </c>
       <c r="I53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2763,7 +2763,7 @@
         <v>1</v>
       </c>
       <c r="L53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>SE3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DSR3</t>
+          <t>DSR1</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2786,19 +2786,19 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>593</v>
+        <v>474.438</v>
       </c>
       <c r="F54" t="n">
         <v>24</v>
       </c>
       <c r="G54" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="H54" t="n">
-        <v>2000</v>
+        <v>150</v>
       </c>
       <c r="I54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
@@ -2807,7 +2807,7 @@
         <v>1</v>
       </c>
       <c r="L54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -2816,12 +2816,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>SE3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2830,7 +2830,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>64.70699999999999</v>
+        <v>474.438</v>
       </c>
       <c r="F55" t="n">
         <v>24</v>
@@ -2839,7 +2839,7 @@
         <v>24</v>
       </c>
       <c r="H55" t="n">
-        <v>150</v>
+        <v>244</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -2860,12 +2860,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>SE3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>DSR2</t>
+          <t>DSR3</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>64.70699999999999</v>
+        <v>474.438</v>
       </c>
       <c r="F56" t="n">
         <v>24</v>
@@ -2883,7 +2883,7 @@
         <v>24</v>
       </c>
       <c r="H56" t="n">
-        <v>244</v>
+        <v>376</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -2904,12 +2904,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SE1</t>
+          <t>SE4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DSR3</t>
+          <t>DSR1</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2918,7 +2918,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>64.70699999999999</v>
+        <v>132.15</v>
       </c>
       <c r="F57" t="n">
         <v>24</v>
@@ -2927,7 +2927,7 @@
         <v>24</v>
       </c>
       <c r="H57" t="n">
-        <v>376</v>
+        <v>150</v>
       </c>
       <c r="I57" t="n">
         <v>1</v>
@@ -2948,12 +2948,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SE2</t>
+          <t>SE4</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>91.36199999999999</v>
+        <v>132.15</v>
       </c>
       <c r="F58" t="n">
         <v>24</v>
@@ -2971,7 +2971,7 @@
         <v>24</v>
       </c>
       <c r="H58" t="n">
-        <v>150</v>
+        <v>244</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
@@ -2992,12 +2992,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SE2</t>
+          <t>SE4</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DSR2</t>
+          <t>DSR3</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3006,7 +3006,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>91.36199999999999</v>
+        <v>132.15</v>
       </c>
       <c r="F59" t="n">
         <v>24</v>
@@ -3015,7 +3015,7 @@
         <v>24</v>
       </c>
       <c r="H59" t="n">
-        <v>244</v>
+        <v>376</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -3036,12 +3036,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SE2</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>DSR3</t>
+          <t>DSR1</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3050,7 +3050,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>91.36199999999999</v>
+        <v>30</v>
       </c>
       <c r="F60" t="n">
         <v>24</v>
@@ -3059,10 +3059,10 @@
         <v>24</v>
       </c>
       <c r="H60" t="n">
-        <v>376</v>
+        <v>400</v>
       </c>
       <c r="I60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SE3</t>
+          <t>UKgb</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3094,19 +3094,19 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>474.438</v>
+        <v>3149.602</v>
       </c>
       <c r="F61" t="n">
         <v>24</v>
       </c>
       <c r="G61" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="H61" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J61" t="n">
         <v>0</v>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SE3</t>
+          <t>UKgb</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3138,19 +3138,19 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>474.438</v>
+        <v>3576.882</v>
       </c>
       <c r="F62" t="n">
         <v>24</v>
       </c>
       <c r="G62" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H62" t="n">
-        <v>244</v>
+        <v>130.21</v>
       </c>
       <c r="I62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -3168,12 +3168,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SE3</t>
+          <t>UKni</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>DSR3</t>
+          <t>DSR1</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3182,16 +3182,16 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>474.438</v>
+        <v>160</v>
       </c>
       <c r="F63" t="n">
         <v>24</v>
       </c>
       <c r="G63" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="H63" t="n">
-        <v>376</v>
+        <v>500</v>
       </c>
       <c r="I63" t="n">
         <v>1</v>
@@ -3203,7 +3203,7 @@
         <v>1</v>
       </c>
       <c r="L63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -3212,12 +3212,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SE4</t>
+          <t>UKni</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DSR1</t>
+          <t>DSR2</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>132.15</v>
+        <v>10</v>
       </c>
       <c r="F64" t="n">
         <v>24</v>
@@ -3235,7 +3235,7 @@
         <v>24</v>
       </c>
       <c r="H64" t="n">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
@@ -3247,314 +3247,6 @@
         <v>1</v>
       </c>
       <c r="L64" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>1</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>SE4</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>DSR2</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>132.15</v>
-      </c>
-      <c r="F65" t="n">
-        <v>24</v>
-      </c>
-      <c r="G65" t="n">
-        <v>24</v>
-      </c>
-      <c r="H65" t="n">
-        <v>244</v>
-      </c>
-      <c r="I65" t="n">
-        <v>1</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" t="n">
-        <v>1</v>
-      </c>
-      <c r="L65" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>1</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>SE4</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>DSR3</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>132.15</v>
-      </c>
-      <c r="F66" t="n">
-        <v>24</v>
-      </c>
-      <c r="G66" t="n">
-        <v>24</v>
-      </c>
-      <c r="H66" t="n">
-        <v>376</v>
-      </c>
-      <c r="I66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" t="n">
-        <v>1</v>
-      </c>
-      <c r="L66" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>1</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>DSR1</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>30</v>
-      </c>
-      <c r="F67" t="n">
-        <v>24</v>
-      </c>
-      <c r="G67" t="n">
-        <v>24</v>
-      </c>
-      <c r="H67" t="n">
-        <v>400</v>
-      </c>
-      <c r="I67" t="n">
-        <v>2</v>
-      </c>
-      <c r="J67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" t="n">
-        <v>1</v>
-      </c>
-      <c r="L67" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>1</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>UKgb</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>DSR1</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>3149.602</v>
-      </c>
-      <c r="F68" t="n">
-        <v>24</v>
-      </c>
-      <c r="G68" t="n">
-        <v>2</v>
-      </c>
-      <c r="H68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I68" t="n">
-        <v>5</v>
-      </c>
-      <c r="J68" t="n">
-        <v>0</v>
-      </c>
-      <c r="K68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L68" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>1</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>UKgb</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>DSR2</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E69" t="n">
-        <v>3576.882</v>
-      </c>
-      <c r="F69" t="n">
-        <v>24</v>
-      </c>
-      <c r="G69" t="n">
-        <v>6</v>
-      </c>
-      <c r="H69" t="n">
-        <v>130.21</v>
-      </c>
-      <c r="I69" t="n">
-        <v>10</v>
-      </c>
-      <c r="J69" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L69" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>1</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>UKni</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>DSR1</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>160</v>
-      </c>
-      <c r="F70" t="n">
-        <v>24</v>
-      </c>
-      <c r="G70" t="n">
-        <v>5</v>
-      </c>
-      <c r="H70" t="n">
-        <v>500</v>
-      </c>
-      <c r="I70" t="n">
-        <v>1</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="n">
-        <v>1</v>
-      </c>
-      <c r="L70" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>1</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>UKni</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>DSR2</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>DSR</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>10</v>
-      </c>
-      <c r="F71" t="n">
-        <v>24</v>
-      </c>
-      <c r="G71" t="n">
-        <v>24</v>
-      </c>
-      <c r="H71" t="n">
-        <v>500</v>
-      </c>
-      <c r="I71" t="n">
-        <v>1</v>
-      </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="n">
-        <v>1</v>
-      </c>
-      <c r="L71" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>